<commit_message>
Dodaj lokalny podglad Leaflet i oddziel publikacje
</commit_message>
<xml_diff>
--- a/routes/rejsy.xlsx
+++ b/routes/rejsy.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Rejsy" sheetId="1" state="visible" r:id="rId1"/>
@@ -338,222 +338,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>tc={6C06E6BA-486A-3D5B-5594-BC1A115D1E43}</author>
-    <author>tc={00149ADD-0244-9303-7045-DB53D8549BE7}</author>
-    <author>tc={0F415041-2C15-BD8F-6121-0224319A01C7}</author>
-    <author>tc={0945DAFB-47DD-E151-3D5A-4A3F87FA4A6D}</author>
-    <author>tc={7056D43C-E51F-7FF2-E984-622B3D539827}</author>
-    <author>tc={44966240-032F-3233-94C2-8A1A0BCB0F6C}</author>
-  </authors>
-  <commentList>
-    <comment ref="A1" authorId="0" shapeId="0">
-      <text>
-        <t>[Komentarz podzielony na wątki]
-Używana wersja programu Excel umożliwia odczytanie tego komentarza podzielonego na wątki, jednak wszelkie wprowadzone w nim zmiany zostaną usunięte po otwarciu pliku w nowszej wersji programu Excel. Dowiedz się więcej: https://go.microsoft.com/fwlink/?linkid=870924
-Komentarz:
-    Wymagane. Unikalny identyfikator rejsu, np. MED-2026-01.</t>
-      </text>
-    </comment>
-    <comment ref="B1" authorId="1" shapeId="0">
-      <text>
-        <t>[Komentarz podzielony na wątki]
-Używana wersja programu Excel umożliwia odczytanie tego komentarza podzielonego na wątki, jednak wszelkie wprowadzone w nim zmiany zostaną usunięte po otwarciu pliku w nowszej wersji programu Excel. Dowiedz się więcej: https://go.microsoft.com/fwlink/?linkid=870924
-Komentarz:
-    Wymagane. Nazwa rejsu widoczna w wynikach i pliku KML.</t>
-      </text>
-    </comment>
-    <comment ref="C1" authorId="2" shapeId="0">
-      <text>
-        <t>[Komentarz podzielony na wątki]
-Używana wersja programu Excel umożliwia odczytanie tego komentarza podzielonego na wątki, jednak wszelkie wprowadzone w nim zmiany zostaną usunięte po otwarciu pliku w nowszej wersji programu Excel. Dowiedz się więcej: https://go.microsoft.com/fwlink/?linkid=870924
-Komentarz:
-    Wymagane. Pierwszy dzień rejsu; jest liczony jako dzień 1.</t>
-      </text>
-    </comment>
-    <comment ref="D1" authorId="3" shapeId="0">
-      <text>
-        <t>[Komentarz podzielony na wątki]
-Używana wersja programu Excel umożliwia odczytanie tego komentarza podzielonego na wątki, jednak wszelkie wprowadzone w nim zmiany zostaną usunięte po otwarciu pliku w nowszej wersji programu Excel. Dowiedz się więcej: https://go.microsoft.com/fwlink/?linkid=870924
-Komentarz:
-    Opcjonalne. Kolor trasy w formacie #RRGGBB. Puste pole oznacza #0057B8.</t>
-      </text>
-    </comment>
-    <comment ref="E1" authorId="4" shapeId="0">
-      <text>
-        <t>[Komentarz podzielony na wątki]
-Używana wersja programu Excel umożliwia odczytanie tego komentarza podzielonego na wątki, jednak wszelkie wprowadzone w nim zmiany zostaną usunięte po otwarciu pliku w nowszej wersji programu Excel. Dowiedz się więcej: https://go.microsoft.com/fwlink/?linkid=870924
-Komentarz:
-    Opcjonalne pole użytkownika. Program zachowuje je bez interpretacji.</t>
-      </text>
-    </comment>
-    <comment ref="F1" authorId="5" shapeId="0">
-      <text>
-        <t>[Komentarz podzielony na wątki]
-Używana wersja programu Excel umożliwia odczytanie tego komentarza podzielonego na wątki, jednak wszelkie wprowadzone w nim zmiany zostaną usunięte po otwarciu pliku w nowszej wersji programu Excel. Dowiedz się więcej: https://go.microsoft.com/fwlink/?linkid=870924
-Komentarz:
-    Opcjonalne notatki dotyczące całego rejsu.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>tc={66ED7548-0EE1-E10A-5A92-E98D52DBF21E}</author>
-    <author>tc={5D261DAC-39FE-089A-E5C8-CD1EA7ED2A3F}</author>
-    <author>tc={0B17727F-53CD-3BA4-5E16-7CEDE9B5D5DC}</author>
-    <author>tc={C1EFCBDE-9761-7763-ACD2-971A733DBB15}</author>
-    <author>tc={1502A828-EB65-E3FF-C1EF-3A995F2B3FA0}</author>
-    <author>tc={98848021-E309-4381-2815-B843730C12D4}</author>
-    <author>tc={F371DF00-DF82-1CB1-AFF2-1147B2F48449}</author>
-    <author>tc={47AAE284-1DAD-1C11-67E3-A688DEEA3584}</author>
-    <author>tc={09E49AB7-A45F-B8EA-2DFA-707F3DE48532}</author>
-  </authors>
-  <commentList>
-    <comment ref="A1" authorId="0" shapeId="0">
-      <text>
-        <t>[Komentarz podzielony na wątki]
-Używana wersja programu Excel umożliwia odczytanie tego komentarza podzielonego na wątki, jednak wszelkie wprowadzone w nim zmiany zostaną usunięte po otwarciu pliku w nowszej wersji programu Excel. Dowiedz się więcej: https://go.microsoft.com/fwlink/?linkid=870924
-Komentarz:
-    Wymagane. Musi odpowiadać identyfikatorowi z arkusza Rejsy.</t>
-      </text>
-    </comment>
-    <comment ref="B1" authorId="1" shapeId="0">
-      <text>
-        <t>[Komentarz podzielony na wątki]
-Używana wersja programu Excel umożliwia odczytanie tego komentarza podzielonego na wątki, jednak wszelkie wprowadzone w nim zmiany zostaną usunięte po otwarciu pliku w nowszej wersji programu Excel. Dowiedz się więcej: https://go.microsoft.com/fwlink/?linkid=870924
-Komentarz:
-    Wymagane. Kolejność portu w rejsie: 1, 2, 3…</t>
-      </text>
-    </comment>
-    <comment ref="C1" authorId="2" shapeId="0">
-      <text>
-        <t>[Komentarz podzielony na wątki]
-Używana wersja programu Excel umożliwia odczytanie tego komentarza podzielonego na wątki, jednak wszelkie wprowadzone w nim zmiany zostaną usunięte po otwarciu pliku w nowszej wersji programu Excel. Dowiedz się więcej: https://go.microsoft.com/fwlink/?linkid=870924
-Komentarz:
-    Wymagane. Nazwa portu.</t>
-      </text>
-    </comment>
-    <comment ref="D1" authorId="3" shapeId="0">
-      <text>
-        <t>[Komentarz podzielony na wątki]
-Używana wersja programu Excel umożliwia odczytanie tego komentarza podzielonego na wątki, jednak wszelkie wprowadzone w nim zmiany zostaną usunięte po otwarciu pliku w nowszej wersji programu Excel. Dowiedz się więcej: https://go.microsoft.com/fwlink/?linkid=870924
-Komentarz:
-    Zalecane. Kraj lub region pomaga jednoznacznie znaleźć port.</t>
-      </text>
-    </comment>
-    <comment ref="E1" authorId="4" shapeId="0">
-      <text>
-        <t>[Komentarz podzielony na wątki]
-Używana wersja programu Excel umożliwia odczytanie tego komentarza podzielonego na wątki, jednak wszelkie wprowadzone w nim zmiany zostaną usunięte po otwarciu pliku w nowszej wersji programu Excel. Dowiedz się więcej: https://go.microsoft.com/fwlink/?linkid=870924
-Komentarz:
-    Wymagane. Wpisz konkretną datę albo +N, np. +4 oznacza wpływ w 4. dniu rejsu.</t>
-      </text>
-    </comment>
-    <comment ref="F1" authorId="5" shapeId="0">
-      <text>
-        <t>[Komentarz podzielony na wątki]
-Używana wersja programu Excel umożliwia odczytanie tego komentarza podzielonego na wątki, jednak wszelkie wprowadzone w nim zmiany zostaną usunięte po otwarciu pliku w nowszej wersji programu Excel. Dowiedz się więcej: https://go.microsoft.com/fwlink/?linkid=870924
-Komentarz:
-    Opcjonalne. Liczba dni postoju. Puste pole oznacza 1; dla startu można wpisać 0.</t>
-      </text>
-    </comment>
-    <comment ref="G1" authorId="6" shapeId="0">
-      <text>
-        <t>[Komentarz podzielony na wątki]
-Używana wersja programu Excel umożliwia odczytanie tego komentarza podzielonego na wątki, jednak wszelkie wprowadzone w nim zmiany zostaną usunięte po otwarciu pliku w nowszej wersji programu Excel. Dowiedz się więcej: https://go.microsoft.com/fwlink/?linkid=870924
-Komentarz:
-    Opcjonalne. Szerokość geograficzna. Lat i Lon należy podać razem.</t>
-      </text>
-    </comment>
-    <comment ref="H1" authorId="7" shapeId="0">
-      <text>
-        <t>[Komentarz podzielony na wątki]
-Używana wersja programu Excel umożliwia odczytanie tego komentarza podzielonego na wątki, jednak wszelkie wprowadzone w nim zmiany zostaną usunięte po otwarciu pliku w nowszej wersji programu Excel. Dowiedz się więcej: https://go.microsoft.com/fwlink/?linkid=870924
-Komentarz:
-    Opcjonalne. Długość geograficzna. Lat i Lon należy podać razem.</t>
-      </text>
-    </comment>
-    <comment ref="I1" authorId="8" shapeId="0">
-      <text>
-        <t>[Komentarz podzielony na wątki]
-Używana wersja programu Excel umożliwia odczytanie tego komentarza podzielonego na wątki, jednak wszelkie wprowadzone w nim zmiany zostaną usunięte po otwarciu pliku w nowszej wersji programu Excel. Dowiedz się więcej: https://go.microsoft.com/fwlink/?linkid=870924
-Komentarz:
-    Opcjonalne notatki dotyczące tego zawinięcia.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment3.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>tc={250D9B77-103F-8F8E-FEDD-740F575904F2}</author>
-    <author>tc={1AF43617-71FE-C117-1EAF-D772CA75A463}</author>
-    <author>tc={8ABB4566-A4D9-9801-27DA-5FC0C80101F8}</author>
-    <author>tc={685A844F-5579-CCCD-963D-A6F078DAACB0}</author>
-    <author>tc={69297FAC-1501-2590-E53C-1F7CF5A78FAD}</author>
-    <author>tc={084E301B-DE47-00A8-7A64-96ED9446E965}</author>
-  </authors>
-  <commentList>
-    <comment ref="A1" authorId="0" shapeId="0">
-      <text>
-        <t>[Komentarz podzielony na wątki]
-Używana wersja programu Excel umożliwia odczytanie tego komentarza podzielonego na wątki, jednak wszelkie wprowadzone w nim zmiany zostaną usunięte po otwarciu pliku w nowszej wersji programu Excel. Dowiedz się więcej: https://go.microsoft.com/fwlink/?linkid=870924
-Komentarz:
-    Arkusz wynikowy. Program generuje jego zawartość na podstawie Rejsy i Porty.</t>
-      </text>
-    </comment>
-    <comment ref="B1" authorId="1" shapeId="0">
-      <text>
-        <t>[Komentarz podzielony na wątki]
-Używana wersja programu Excel umożliwia odczytanie tego komentarza podzielonego na wątki, jednak wszelkie wprowadzone w nim zmiany zostaną usunięte po otwarciu pliku w nowszej wersji programu Excel. Dowiedz się więcej: https://go.microsoft.com/fwlink/?linkid=870924
-Komentarz:
-    Numer kolejnego etapu w obrębie rejsu.</t>
-      </text>
-    </comment>
-    <comment ref="F1" authorId="2" shapeId="0">
-      <text>
-        <t>[Komentarz podzielony na wątki]
-Używana wersja programu Excel umożliwia odczytanie tego komentarza podzielonego na wątki, jednak wszelkie wprowadzone w nim zmiany zostaną usunięte po otwarciu pliku w nowszej wersji programu Excel. Dowiedz się więcej: https://go.microsoft.com/fwlink/?linkid=870924
-Komentarz:
-    Pierwszy dzień etapu, po uwzględnieniu postoju w porcie początkowym.</t>
-      </text>
-    </comment>
-    <comment ref="G1" authorId="3" shapeId="0">
-      <text>
-        <t>[Komentarz podzielony na wątki]
-Używana wersja programu Excel umożliwia odczytanie tego komentarza podzielonego na wątki, jednak wszelkie wprowadzone w nim zmiany zostaną usunięte po otwarciu pliku w nowszej wersji programu Excel. Dowiedz się więcej: https://go.microsoft.com/fwlink/?linkid=870924
-Komentarz:
-    Dzień wpływu do portu końcowego.</t>
-      </text>
-    </comment>
-    <comment ref="L1" authorId="4" shapeId="0">
-      <text>
-        <t>[Komentarz podzielony na wątki]
-Używana wersja programu Excel umożliwia odczytanie tego komentarza podzielonego na wątki, jednak wszelkie wprowadzone w nim zmiany zostaną usunięte po otwarciu pliku w nowszej wersji programu Excel. Dowiedz się więcej: https://go.microsoft.com/fwlink/?linkid=870924
-Komentarz:
-    Dystans morskiej trasy w milach morskich, jeśli zwróci go sea-router.</t>
-      </text>
-    </comment>
-    <comment ref="N1" authorId="5" shapeId="0">
-      <text>
-        <t>[Komentarz podzielony na wątki]
-Używana wersja programu Excel umożliwia odczytanie tego komentarza podzielonego na wątki, jednak wszelkie wprowadzone w nim zmiany zostaną usunięte po otwarciu pliku w nowszej wersji programu Excel. Dowiedz się więcej: https://go.microsoft.com/fwlink/?linkid=870924
-Komentarz:
-    Stan przetwarzania etapu, np. gotowy lub brak_trasy.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RejsyTable" displayName="RejsyTable" ref="A1:F3" headerRowCount="1" totalsRowShown="0">
   <autoFilter ref="A1:F3"/>
@@ -570,8 +354,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PortyTable" displayName="PortyTable" ref="A1:I4" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A1:I4"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PortyTable" displayName="PortyTable" ref="A1:I10" headerRowCount="1" totalsRowShown="0">
+  <autoFilter ref="A1:I10"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Rejs_ID"/>
     <tableColumn id="2" name="Kolejnosc"/>
@@ -588,7 +372,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="EtapyTable" displayName="EtapyTable" ref="A1:O3" headerRowCount="1" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="EtapyTable" displayName="EtapyTable" ref="A1:O9" headerRowCount="1" insertRow="1" totalsRowShown="0">
   <autoFilter ref="A1:O2"/>
   <tableColumns count="15">
     <tableColumn id="1" name="Rejs_ID"/>
@@ -1684,7 +1468,6 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
@@ -1697,7 +1480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I495"/>
+  <dimension ref="A1:I501"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1771,7 +1554,11 @@
           <t>Triest</t>
         </is>
       </c>
-      <c r="D2" s="4" t="n"/>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>Włochy</t>
+        </is>
+      </c>
       <c r="E2" s="31" t="n">
         <v>45633</v>
       </c>
@@ -1796,7 +1583,11 @@
           <t>Dubrownik</t>
         </is>
       </c>
-      <c r="D3" s="34" t="n"/>
+      <c r="D3" s="34" t="inlineStr">
+        <is>
+          <t>Chorwacja</t>
+        </is>
+      </c>
       <c r="E3" s="35" t="n">
         <v>1</v>
       </c>
@@ -1821,7 +1612,11 @@
           <t>Katania</t>
         </is>
       </c>
-      <c r="D4" s="34" t="n"/>
+      <c r="D4" s="34" t="inlineStr">
+        <is>
+          <t>Włochy</t>
+        </is>
+      </c>
       <c r="E4" s="38" t="n">
         <v>45636</v>
       </c>
@@ -1837,70 +1632,178 @@
       <c r="I4" s="37" t="n"/>
     </row>
     <row r="5" ht="21.95" customHeight="1">
-      <c r="A5" s="7" t="n"/>
-      <c r="B5" s="15" t="n"/>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="5" t="n"/>
-      <c r="E5" s="11" t="n"/>
-      <c r="F5" s="15" t="n"/>
-      <c r="G5" s="17" t="n"/>
-      <c r="H5" s="17" t="n"/>
-      <c r="I5" s="13" t="n"/>
+      <c r="A5" s="32" t="n"/>
+      <c r="B5" s="33" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="34" t="inlineStr">
+        <is>
+          <t>Civitavecchia</t>
+        </is>
+      </c>
+      <c r="D5" s="34" t="inlineStr">
+        <is>
+          <t>Włochy</t>
+        </is>
+      </c>
+      <c r="E5" s="35" t="n">
+        <v>4</v>
+      </c>
+      <c r="F5" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" s="36" t="n">
+        <v>42.0937524</v>
+      </c>
+      <c r="H5" s="36" t="n">
+        <v>11.7922462</v>
+      </c>
+      <c r="I5" s="37" t="n"/>
     </row>
     <row r="6" ht="21.95" customHeight="1">
-      <c r="A6" s="7" t="n"/>
-      <c r="B6" s="15" t="n"/>
-      <c r="C6" s="5" t="n"/>
-      <c r="D6" s="5" t="n"/>
-      <c r="E6" s="11" t="n"/>
-      <c r="F6" s="15" t="n"/>
-      <c r="G6" s="17" t="n"/>
-      <c r="H6" s="17" t="n"/>
-      <c r="I6" s="13" t="n"/>
+      <c r="A6" s="32" t="n"/>
+      <c r="B6" s="33" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="34" t="inlineStr">
+        <is>
+          <t>Savona</t>
+        </is>
+      </c>
+      <c r="D6" s="34" t="inlineStr">
+        <is>
+          <t>Włochy</t>
+        </is>
+      </c>
+      <c r="E6" s="35" t="n">
+        <v>5</v>
+      </c>
+      <c r="F6" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" s="36" t="n">
+        <v>44.3080251</v>
+      </c>
+      <c r="H6" s="36" t="n">
+        <v>8.4810315</v>
+      </c>
+      <c r="I6" s="37" t="n"/>
     </row>
     <row r="7" ht="21.95" customHeight="1">
-      <c r="A7" s="7" t="n"/>
-      <c r="B7" s="15" t="n"/>
-      <c r="C7" s="5" t="n"/>
-      <c r="D7" s="5" t="n"/>
-      <c r="E7" s="11" t="n"/>
-      <c r="F7" s="15" t="n"/>
-      <c r="G7" s="17" t="n"/>
-      <c r="H7" s="17" t="n"/>
-      <c r="I7" s="13" t="n"/>
+      <c r="A7" s="32" t="n"/>
+      <c r="B7" s="33" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" s="34" t="inlineStr">
+        <is>
+          <t>Marsylia</t>
+        </is>
+      </c>
+      <c r="D7" s="34" t="inlineStr">
+        <is>
+          <t>Francja</t>
+        </is>
+      </c>
+      <c r="E7" s="35" t="n">
+        <v>6</v>
+      </c>
+      <c r="F7" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="36" t="n">
+        <v>43.2963986</v>
+      </c>
+      <c r="H7" s="36" t="n">
+        <v>5.3777888</v>
+      </c>
+      <c r="I7" s="37" t="n"/>
     </row>
     <row r="8" ht="21.95" customHeight="1">
-      <c r="A8" s="7" t="n"/>
-      <c r="B8" s="15" t="n"/>
-      <c r="C8" s="5" t="n"/>
-      <c r="D8" s="5" t="n"/>
-      <c r="E8" s="11" t="n"/>
-      <c r="F8" s="15" t="n"/>
-      <c r="G8" s="17" t="n"/>
-      <c r="H8" s="17" t="n"/>
-      <c r="I8" s="13" t="n"/>
+      <c r="A8" s="32" t="n"/>
+      <c r="B8" s="33" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" s="34" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="D8" s="34" t="inlineStr">
+        <is>
+          <t>Hiszpania</t>
+        </is>
+      </c>
+      <c r="E8" s="35" t="n">
+        <v>7</v>
+      </c>
+      <c r="F8" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="36" t="n">
+        <v>41.3825802</v>
+      </c>
+      <c r="H8" s="36" t="n">
+        <v>2.177073</v>
+      </c>
+      <c r="I8" s="37" t="n"/>
     </row>
     <row r="9" ht="21.95" customHeight="1">
-      <c r="A9" s="7" t="n"/>
-      <c r="B9" s="15" t="n"/>
-      <c r="C9" s="5" t="n"/>
-      <c r="D9" s="5" t="n"/>
-      <c r="E9" s="11" t="n"/>
-      <c r="F9" s="15" t="n"/>
-      <c r="G9" s="17" t="n"/>
-      <c r="H9" s="17" t="n"/>
-      <c r="I9" s="13" t="n"/>
+      <c r="A9" s="32" t="n"/>
+      <c r="B9" s="33" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" s="34" t="inlineStr">
+        <is>
+          <t>Casablanca</t>
+        </is>
+      </c>
+      <c r="D9" s="34" t="inlineStr">
+        <is>
+          <t>Maroko</t>
+        </is>
+      </c>
+      <c r="E9" s="35" t="n">
+        <v>10</v>
+      </c>
+      <c r="F9" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="36" t="n">
+        <v>33.5945144</v>
+      </c>
+      <c r="H9" s="36" t="n">
+        <v>-7.6200284</v>
+      </c>
+      <c r="I9" s="37" t="n"/>
     </row>
     <row r="10" ht="21.95" customHeight="1">
-      <c r="A10" s="7" t="n"/>
-      <c r="B10" s="15" t="n"/>
-      <c r="C10" s="5" t="n"/>
-      <c r="D10" s="5" t="n"/>
-      <c r="E10" s="11" t="n"/>
-      <c r="F10" s="15" t="n"/>
-      <c r="G10" s="17" t="n"/>
-      <c r="H10" s="17" t="n"/>
-      <c r="I10" s="13" t="n"/>
+      <c r="A10" s="32" t="n"/>
+      <c r="B10" s="33" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" s="34" t="inlineStr">
+        <is>
+          <t>Las Palmas</t>
+        </is>
+      </c>
+      <c r="D10" s="34" t="inlineStr">
+        <is>
+          <t>Hiszpania</t>
+        </is>
+      </c>
+      <c r="E10" s="35" t="n">
+        <v>12</v>
+      </c>
+      <c r="F10" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" s="36" t="n">
+        <v>28.1288694</v>
+      </c>
+      <c r="H10" s="36" t="n">
+        <v>-15.4349015</v>
+      </c>
+      <c r="I10" s="37" t="n"/>
     </row>
     <row r="11" ht="21.95" customHeight="1">
       <c r="A11" s="7" t="n"/>
@@ -7237,33 +7140,92 @@
       <c r="H495" s="17" t="n"/>
       <c r="I495" s="13" t="n"/>
     </row>
-    <row r="496" ht="21.95" customHeight="1"/>
-    <row r="497" ht="21.95" customHeight="1"/>
-    <row r="498" ht="21.95" customHeight="1"/>
-    <row r="499" ht="21.95" customHeight="1"/>
-    <row r="500" ht="21.95" customHeight="1"/>
-    <row r="501" ht="21.95" customHeight="1"/>
+    <row r="496" ht="21.95" customHeight="1">
+      <c r="A496" s="7" t="n"/>
+      <c r="B496" s="15" t="n"/>
+      <c r="C496" s="5" t="n"/>
+      <c r="D496" s="5" t="n"/>
+      <c r="E496" s="11" t="n"/>
+      <c r="F496" s="15" t="n"/>
+      <c r="G496" s="17" t="n"/>
+      <c r="H496" s="17" t="n"/>
+      <c r="I496" s="13" t="n"/>
+    </row>
+    <row r="497" ht="21.95" customHeight="1">
+      <c r="A497" s="7" t="n"/>
+      <c r="B497" s="15" t="n"/>
+      <c r="C497" s="5" t="n"/>
+      <c r="D497" s="5" t="n"/>
+      <c r="E497" s="11" t="n"/>
+      <c r="F497" s="15" t="n"/>
+      <c r="G497" s="17" t="n"/>
+      <c r="H497" s="17" t="n"/>
+      <c r="I497" s="13" t="n"/>
+    </row>
+    <row r="498" ht="21.95" customHeight="1">
+      <c r="A498" s="7" t="n"/>
+      <c r="B498" s="15" t="n"/>
+      <c r="C498" s="5" t="n"/>
+      <c r="D498" s="5" t="n"/>
+      <c r="E498" s="11" t="n"/>
+      <c r="F498" s="15" t="n"/>
+      <c r="G498" s="17" t="n"/>
+      <c r="H498" s="17" t="n"/>
+      <c r="I498" s="13" t="n"/>
+    </row>
+    <row r="499" ht="21.95" customHeight="1">
+      <c r="A499" s="7" t="n"/>
+      <c r="B499" s="15" t="n"/>
+      <c r="C499" s="5" t="n"/>
+      <c r="D499" s="5" t="n"/>
+      <c r="E499" s="11" t="n"/>
+      <c r="F499" s="15" t="n"/>
+      <c r="G499" s="17" t="n"/>
+      <c r="H499" s="17" t="n"/>
+      <c r="I499" s="13" t="n"/>
+    </row>
+    <row r="500" ht="21.95" customHeight="1">
+      <c r="A500" s="7" t="n"/>
+      <c r="B500" s="15" t="n"/>
+      <c r="C500" s="5" t="n"/>
+      <c r="D500" s="5" t="n"/>
+      <c r="E500" s="11" t="n"/>
+      <c r="F500" s="15" t="n"/>
+      <c r="G500" s="17" t="n"/>
+      <c r="H500" s="17" t="n"/>
+      <c r="I500" s="13" t="n"/>
+    </row>
+    <row r="501" ht="21.95" customHeight="1">
+      <c r="A501" s="7" t="n"/>
+      <c r="B501" s="15" t="n"/>
+      <c r="C501" s="5" t="n"/>
+      <c r="D501" s="5" t="n"/>
+      <c r="E501" s="11" t="n"/>
+      <c r="F501" s="15" t="n"/>
+      <c r="G501" s="17" t="n"/>
+      <c r="H501" s="17" t="n"/>
+      <c r="I501" s="13" t="n"/>
+    </row>
   </sheetData>
   <dataValidations count="4">
-    <dataValidation sqref="B2:B495" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="whole">
+    <dataValidation sqref="B2:B501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="whole">
       <formula1>1</formula1>
       <formula2>1000</formula2>
     </dataValidation>
-    <dataValidation sqref="F2:F495" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="whole">
+    <dataValidation sqref="F2:F501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="whole">
       <formula1>0</formula1>
       <formula2>365</formula2>
     </dataValidation>
-    <dataValidation sqref="G2:G495" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="decimal">
+    <dataValidation sqref="G2:G501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="decimal">
       <formula1>-90</formula1>
       <formula2>90</formula2>
     </dataValidation>
-    <dataValidation sqref="H2:H495" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="decimal">
+    <dataValidation sqref="H2:H501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="decimal">
       <formula1>-180</formula1>
       <formula2>180</formula2>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
@@ -7276,7 +7238,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O501"/>
+  <dimension ref="A1:O494"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -7493,105 +7455,369 @@
       <c r="O3" s="26" t="n"/>
     </row>
     <row r="4" ht="21.95" customHeight="1">
-      <c r="A4" s="19" t="n"/>
-      <c r="B4" s="21" t="n"/>
-      <c r="C4" s="19" t="n"/>
-      <c r="D4" s="19" t="n"/>
-      <c r="E4" s="26" t="n"/>
-      <c r="F4" s="27" t="n"/>
-      <c r="G4" s="27" t="n"/>
-      <c r="H4" s="28" t="n"/>
-      <c r="I4" s="28" t="n"/>
-      <c r="J4" s="26" t="n"/>
-      <c r="K4" s="26" t="n"/>
-      <c r="L4" s="29" t="n"/>
-      <c r="M4" s="26" t="n"/>
-      <c r="N4" s="26" t="n"/>
+      <c r="A4" s="19" t="inlineStr">
+        <is>
+          <t>Rejs 3</t>
+        </is>
+      </c>
+      <c r="B4" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="19" t="inlineStr">
+        <is>
+          <t>Katania</t>
+        </is>
+      </c>
+      <c r="D4" s="19" t="inlineStr">
+        <is>
+          <t>Civitavecchia</t>
+        </is>
+      </c>
+      <c r="E4" s="26" t="inlineStr">
+        <is>
+          <t>Katania → Civitavecchia</t>
+        </is>
+      </c>
+      <c r="F4" s="27" t="n">
+        <v>5</v>
+      </c>
+      <c r="G4" s="27" t="n">
+        <v>5</v>
+      </c>
+      <c r="H4" s="28" t="n">
+        <v>45637</v>
+      </c>
+      <c r="I4" s="28" t="n">
+        <v>45637</v>
+      </c>
+      <c r="J4" s="26" t="inlineStr">
+        <is>
+          <t>Dni 5–5</t>
+        </is>
+      </c>
+      <c r="K4" s="26" t="inlineStr">
+        <is>
+          <t>2024-12-11 – 2024-12-11</t>
+        </is>
+      </c>
+      <c r="L4" s="29" t="n">
+        <v>354.6</v>
+      </c>
+      <c r="M4" s="26" t="inlineStr">
+        <is>
+          <t>Rejs-3\geojson\03-Katania-Civitavecchia.geojson</t>
+        </is>
+      </c>
+      <c r="N4" s="26" t="inlineStr">
+        <is>
+          <t>gotowy</t>
+        </is>
+      </c>
       <c r="O4" s="26" t="n"/>
     </row>
     <row r="5" ht="21.95" customHeight="1">
-      <c r="A5" s="19" t="n"/>
-      <c r="B5" s="21" t="n"/>
-      <c r="C5" s="19" t="n"/>
-      <c r="D5" s="19" t="n"/>
-      <c r="E5" s="26" t="n"/>
-      <c r="F5" s="27" t="n"/>
-      <c r="G5" s="27" t="n"/>
-      <c r="H5" s="28" t="n"/>
-      <c r="I5" s="28" t="n"/>
-      <c r="J5" s="26" t="n"/>
-      <c r="K5" s="26" t="n"/>
-      <c r="L5" s="29" t="n"/>
-      <c r="M5" s="26" t="n"/>
-      <c r="N5" s="26" t="n"/>
+      <c r="A5" s="19" t="inlineStr">
+        <is>
+          <t>Rejs 3</t>
+        </is>
+      </c>
+      <c r="B5" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="19" t="inlineStr">
+        <is>
+          <t>Civitavecchia</t>
+        </is>
+      </c>
+      <c r="D5" s="19" t="inlineStr">
+        <is>
+          <t>Savona</t>
+        </is>
+      </c>
+      <c r="E5" s="26" t="inlineStr">
+        <is>
+          <t>Civitavecchia → Savona</t>
+        </is>
+      </c>
+      <c r="F5" s="27" t="n">
+        <v>6</v>
+      </c>
+      <c r="G5" s="27" t="n">
+        <v>6</v>
+      </c>
+      <c r="H5" s="28" t="n">
+        <v>45638</v>
+      </c>
+      <c r="I5" s="28" t="n">
+        <v>45638</v>
+      </c>
+      <c r="J5" s="26" t="inlineStr">
+        <is>
+          <t>Dni 6–6</t>
+        </is>
+      </c>
+      <c r="K5" s="26" t="inlineStr">
+        <is>
+          <t>2024-12-12 – 2024-12-12</t>
+        </is>
+      </c>
+      <c r="L5" s="29" t="n">
+        <v>201.3</v>
+      </c>
+      <c r="M5" s="26" t="inlineStr">
+        <is>
+          <t>Rejs-3\geojson\04-Civitavecchia-Savona.geojson</t>
+        </is>
+      </c>
+      <c r="N5" s="26" t="inlineStr">
+        <is>
+          <t>gotowy</t>
+        </is>
+      </c>
       <c r="O5" s="26" t="n"/>
     </row>
     <row r="6" ht="21.95" customHeight="1">
-      <c r="A6" s="19" t="n"/>
-      <c r="B6" s="21" t="n"/>
-      <c r="C6" s="19" t="n"/>
-      <c r="D6" s="19" t="n"/>
-      <c r="E6" s="26" t="n"/>
-      <c r="F6" s="27" t="n"/>
-      <c r="G6" s="27" t="n"/>
-      <c r="H6" s="28" t="n"/>
-      <c r="I6" s="28" t="n"/>
-      <c r="J6" s="26" t="n"/>
-      <c r="K6" s="26" t="n"/>
-      <c r="L6" s="29" t="n"/>
-      <c r="M6" s="26" t="n"/>
-      <c r="N6" s="26" t="n"/>
+      <c r="A6" s="19" t="inlineStr">
+        <is>
+          <t>Rejs 3</t>
+        </is>
+      </c>
+      <c r="B6" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="19" t="inlineStr">
+        <is>
+          <t>Savona</t>
+        </is>
+      </c>
+      <c r="D6" s="19" t="inlineStr">
+        <is>
+          <t>Marsylia</t>
+        </is>
+      </c>
+      <c r="E6" s="26" t="inlineStr">
+        <is>
+          <t>Savona → Marsylia</t>
+        </is>
+      </c>
+      <c r="F6" s="27" t="n">
+        <v>7</v>
+      </c>
+      <c r="G6" s="27" t="n">
+        <v>7</v>
+      </c>
+      <c r="H6" s="28" t="n">
+        <v>45639</v>
+      </c>
+      <c r="I6" s="28" t="n">
+        <v>45639</v>
+      </c>
+      <c r="J6" s="26" t="inlineStr">
+        <is>
+          <t>Dni 7–7</t>
+        </is>
+      </c>
+      <c r="K6" s="26" t="inlineStr">
+        <is>
+          <t>2024-12-13 – 2024-12-13</t>
+        </is>
+      </c>
+      <c r="L6" s="29" t="n">
+        <v>198.2</v>
+      </c>
+      <c r="M6" s="26" t="inlineStr">
+        <is>
+          <t>Rejs-3\geojson\05-Savona-Marsylia.geojson</t>
+        </is>
+      </c>
+      <c r="N6" s="26" t="inlineStr">
+        <is>
+          <t>gotowy</t>
+        </is>
+      </c>
       <c r="O6" s="26" t="n"/>
     </row>
     <row r="7" ht="21.95" customHeight="1">
-      <c r="A7" s="19" t="n"/>
-      <c r="B7" s="21" t="n"/>
-      <c r="C7" s="19" t="n"/>
-      <c r="D7" s="19" t="n"/>
-      <c r="E7" s="26" t="n"/>
-      <c r="F7" s="27" t="n"/>
-      <c r="G7" s="27" t="n"/>
-      <c r="H7" s="28" t="n"/>
-      <c r="I7" s="28" t="n"/>
-      <c r="J7" s="26" t="n"/>
-      <c r="K7" s="26" t="n"/>
-      <c r="L7" s="29" t="n"/>
-      <c r="M7" s="26" t="n"/>
-      <c r="N7" s="26" t="n"/>
+      <c r="A7" s="19" t="inlineStr">
+        <is>
+          <t>Rejs 3</t>
+        </is>
+      </c>
+      <c r="B7" s="21" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" s="19" t="inlineStr">
+        <is>
+          <t>Marsylia</t>
+        </is>
+      </c>
+      <c r="D7" s="19" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="E7" s="26" t="inlineStr">
+        <is>
+          <t>Marsylia → Barcelona</t>
+        </is>
+      </c>
+      <c r="F7" s="27" t="n">
+        <v>8</v>
+      </c>
+      <c r="G7" s="27" t="n">
+        <v>8</v>
+      </c>
+      <c r="H7" s="28" t="n">
+        <v>45640</v>
+      </c>
+      <c r="I7" s="28" t="n">
+        <v>45640</v>
+      </c>
+      <c r="J7" s="26" t="inlineStr">
+        <is>
+          <t>Dni 8–8</t>
+        </is>
+      </c>
+      <c r="K7" s="26" t="inlineStr">
+        <is>
+          <t>2024-12-14 – 2024-12-14</t>
+        </is>
+      </c>
+      <c r="L7" s="29" t="n">
+        <v>190</v>
+      </c>
+      <c r="M7" s="26" t="inlineStr">
+        <is>
+          <t>Rejs-3\geojson\06-Marsylia-Barcelona.geojson</t>
+        </is>
+      </c>
+      <c r="N7" s="26" t="inlineStr">
+        <is>
+          <t>gotowy</t>
+        </is>
+      </c>
       <c r="O7" s="26" t="n"/>
     </row>
     <row r="8" ht="21.95" customHeight="1">
-      <c r="A8" s="19" t="n"/>
-      <c r="B8" s="21" t="n"/>
-      <c r="C8" s="19" t="n"/>
-      <c r="D8" s="19" t="n"/>
-      <c r="E8" s="26" t="n"/>
-      <c r="F8" s="27" t="n"/>
-      <c r="G8" s="27" t="n"/>
-      <c r="H8" s="28" t="n"/>
-      <c r="I8" s="28" t="n"/>
-      <c r="J8" s="26" t="n"/>
-      <c r="K8" s="26" t="n"/>
-      <c r="L8" s="29" t="n"/>
-      <c r="M8" s="26" t="n"/>
-      <c r="N8" s="26" t="n"/>
+      <c r="A8" s="19" t="inlineStr">
+        <is>
+          <t>Rejs 3</t>
+        </is>
+      </c>
+      <c r="B8" s="21" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" s="19" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="D8" s="19" t="inlineStr">
+        <is>
+          <t>Casablanca</t>
+        </is>
+      </c>
+      <c r="E8" s="26" t="inlineStr">
+        <is>
+          <t>Barcelona → Casablanca</t>
+        </is>
+      </c>
+      <c r="F8" s="27" t="n">
+        <v>9</v>
+      </c>
+      <c r="G8" s="27" t="n">
+        <v>11</v>
+      </c>
+      <c r="H8" s="28" t="n">
+        <v>45641</v>
+      </c>
+      <c r="I8" s="28" t="n">
+        <v>45643</v>
+      </c>
+      <c r="J8" s="26" t="inlineStr">
+        <is>
+          <t>Dni 9–11</t>
+        </is>
+      </c>
+      <c r="K8" s="26" t="inlineStr">
+        <is>
+          <t>2024-12-15 – 2024-12-17</t>
+        </is>
+      </c>
+      <c r="L8" s="29" t="n">
+        <v>731.9</v>
+      </c>
+      <c r="M8" s="26" t="inlineStr">
+        <is>
+          <t>Rejs-3\geojson\07-Barcelona-Casablanca.geojson</t>
+        </is>
+      </c>
+      <c r="N8" s="26" t="inlineStr">
+        <is>
+          <t>gotowy</t>
+        </is>
+      </c>
       <c r="O8" s="26" t="n"/>
     </row>
     <row r="9" ht="21.95" customHeight="1">
-      <c r="A9" s="19" t="n"/>
-      <c r="B9" s="21" t="n"/>
-      <c r="C9" s="19" t="n"/>
-      <c r="D9" s="19" t="n"/>
-      <c r="E9" s="26" t="n"/>
-      <c r="F9" s="27" t="n"/>
-      <c r="G9" s="27" t="n"/>
-      <c r="H9" s="28" t="n"/>
-      <c r="I9" s="28" t="n"/>
-      <c r="J9" s="26" t="n"/>
-      <c r="K9" s="26" t="n"/>
-      <c r="L9" s="29" t="n"/>
-      <c r="M9" s="26" t="n"/>
-      <c r="N9" s="26" t="n"/>
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>Rejs 3</t>
+        </is>
+      </c>
+      <c r="B9" s="21" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" s="19" t="inlineStr">
+        <is>
+          <t>Casablanca</t>
+        </is>
+      </c>
+      <c r="D9" s="19" t="inlineStr">
+        <is>
+          <t>Las Palmas</t>
+        </is>
+      </c>
+      <c r="E9" s="26" t="inlineStr">
+        <is>
+          <t>Casablanca → Las Palmas</t>
+        </is>
+      </c>
+      <c r="F9" s="27" t="n">
+        <v>12</v>
+      </c>
+      <c r="G9" s="27" t="n">
+        <v>13</v>
+      </c>
+      <c r="H9" s="28" t="n">
+        <v>45644</v>
+      </c>
+      <c r="I9" s="28" t="n">
+        <v>45645</v>
+      </c>
+      <c r="J9" s="26" t="inlineStr">
+        <is>
+          <t>Dni 12–13</t>
+        </is>
+      </c>
+      <c r="K9" s="26" t="inlineStr">
+        <is>
+          <t>2024-12-18 – 2024-12-19</t>
+        </is>
+      </c>
+      <c r="L9" s="29" t="n">
+        <v>538.5</v>
+      </c>
+      <c r="M9" s="26" t="inlineStr">
+        <is>
+          <t>Rejs-3\geojson\08-Casablanca-Las-Palmas.geojson</t>
+        </is>
+      </c>
+      <c r="N9" s="26" t="inlineStr">
+        <is>
+          <t>gotowy</t>
+        </is>
+      </c>
       <c r="O9" s="26" t="n"/>
     </row>
     <row r="10" ht="21.95" customHeight="1">
@@ -15839,128 +16065,8 @@
       <c r="N494" s="26" t="n"/>
       <c r="O494" s="26" t="n"/>
     </row>
-    <row r="495" ht="21.95" customHeight="1">
-      <c r="A495" s="19" t="n"/>
-      <c r="B495" s="21" t="n"/>
-      <c r="C495" s="19" t="n"/>
-      <c r="D495" s="19" t="n"/>
-      <c r="E495" s="26" t="n"/>
-      <c r="F495" s="27" t="n"/>
-      <c r="G495" s="27" t="n"/>
-      <c r="H495" s="28" t="n"/>
-      <c r="I495" s="28" t="n"/>
-      <c r="J495" s="26" t="n"/>
-      <c r="K495" s="26" t="n"/>
-      <c r="L495" s="29" t="n"/>
-      <c r="M495" s="26" t="n"/>
-      <c r="N495" s="26" t="n"/>
-      <c r="O495" s="26" t="n"/>
-    </row>
-    <row r="496" ht="21.95" customHeight="1">
-      <c r="A496" s="19" t="n"/>
-      <c r="B496" s="21" t="n"/>
-      <c r="C496" s="19" t="n"/>
-      <c r="D496" s="19" t="n"/>
-      <c r="E496" s="26" t="n"/>
-      <c r="F496" s="27" t="n"/>
-      <c r="G496" s="27" t="n"/>
-      <c r="H496" s="28" t="n"/>
-      <c r="I496" s="28" t="n"/>
-      <c r="J496" s="26" t="n"/>
-      <c r="K496" s="26" t="n"/>
-      <c r="L496" s="29" t="n"/>
-      <c r="M496" s="26" t="n"/>
-      <c r="N496" s="26" t="n"/>
-      <c r="O496" s="26" t="n"/>
-    </row>
-    <row r="497" ht="21.95" customHeight="1">
-      <c r="A497" s="19" t="n"/>
-      <c r="B497" s="21" t="n"/>
-      <c r="C497" s="19" t="n"/>
-      <c r="D497" s="19" t="n"/>
-      <c r="E497" s="26" t="n"/>
-      <c r="F497" s="27" t="n"/>
-      <c r="G497" s="27" t="n"/>
-      <c r="H497" s="28" t="n"/>
-      <c r="I497" s="28" t="n"/>
-      <c r="J497" s="26" t="n"/>
-      <c r="K497" s="26" t="n"/>
-      <c r="L497" s="29" t="n"/>
-      <c r="M497" s="26" t="n"/>
-      <c r="N497" s="26" t="n"/>
-      <c r="O497" s="26" t="n"/>
-    </row>
-    <row r="498" ht="21.95" customHeight="1">
-      <c r="A498" s="19" t="n"/>
-      <c r="B498" s="21" t="n"/>
-      <c r="C498" s="19" t="n"/>
-      <c r="D498" s="19" t="n"/>
-      <c r="E498" s="26" t="n"/>
-      <c r="F498" s="27" t="n"/>
-      <c r="G498" s="27" t="n"/>
-      <c r="H498" s="28" t="n"/>
-      <c r="I498" s="28" t="n"/>
-      <c r="J498" s="26" t="n"/>
-      <c r="K498" s="26" t="n"/>
-      <c r="L498" s="29" t="n"/>
-      <c r="M498" s="26" t="n"/>
-      <c r="N498" s="26" t="n"/>
-      <c r="O498" s="26" t="n"/>
-    </row>
-    <row r="499" ht="21.95" customHeight="1">
-      <c r="A499" s="19" t="n"/>
-      <c r="B499" s="21" t="n"/>
-      <c r="C499" s="19" t="n"/>
-      <c r="D499" s="19" t="n"/>
-      <c r="E499" s="26" t="n"/>
-      <c r="F499" s="27" t="n"/>
-      <c r="G499" s="27" t="n"/>
-      <c r="H499" s="28" t="n"/>
-      <c r="I499" s="28" t="n"/>
-      <c r="J499" s="26" t="n"/>
-      <c r="K499" s="26" t="n"/>
-      <c r="L499" s="29" t="n"/>
-      <c r="M499" s="26" t="n"/>
-      <c r="N499" s="26" t="n"/>
-      <c r="O499" s="26" t="n"/>
-    </row>
-    <row r="500" ht="21.95" customHeight="1">
-      <c r="A500" s="19" t="n"/>
-      <c r="B500" s="21" t="n"/>
-      <c r="C500" s="19" t="n"/>
-      <c r="D500" s="19" t="n"/>
-      <c r="E500" s="26" t="n"/>
-      <c r="F500" s="27" t="n"/>
-      <c r="G500" s="27" t="n"/>
-      <c r="H500" s="28" t="n"/>
-      <c r="I500" s="28" t="n"/>
-      <c r="J500" s="26" t="n"/>
-      <c r="K500" s="26" t="n"/>
-      <c r="L500" s="29" t="n"/>
-      <c r="M500" s="26" t="n"/>
-      <c r="N500" s="26" t="n"/>
-      <c r="O500" s="26" t="n"/>
-    </row>
-    <row r="501" ht="21.95" customHeight="1">
-      <c r="A501" s="19" t="n"/>
-      <c r="B501" s="21" t="n"/>
-      <c r="C501" s="19" t="n"/>
-      <c r="D501" s="19" t="n"/>
-      <c r="E501" s="26" t="n"/>
-      <c r="F501" s="27" t="n"/>
-      <c r="G501" s="27" t="n"/>
-      <c r="H501" s="28" t="n"/>
-      <c r="I501" s="28" t="n"/>
-      <c r="J501" s="26" t="n"/>
-      <c r="K501" s="26" t="n"/>
-      <c r="L501" s="29" t="n"/>
-      <c r="M501" s="26" t="n"/>
-      <c r="N501" s="26" t="n"/>
-      <c r="O501" s="26" t="n"/>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>

</xml_diff>